<commit_message>
feat: pdf reader used
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs - deitado.xlsx
+++ b/08 - Excels/Open-LPs - deitado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED98AC8-90D3-420B-A156-B125C18776F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3D5295-EFE7-41D4-99C5-BD27718B2F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,6 +88,9 @@
     <t>LP-051682</t>
   </si>
   <si>
+    <t>LP-051635</t>
+  </si>
+  <si>
     <t>LP-051709</t>
   </si>
   <si>
@@ -220,9 +223,6 @@
     <t>LP-051683</t>
   </si>
   <si>
-    <t>LP-051685</t>
-  </si>
-  <si>
     <t>LP-051903</t>
   </si>
   <si>
@@ -247,7 +247,7 @@
     <t>LP-052148</t>
   </si>
   <si>
-    <t>LP-052262</t>
+    <t>LP-052462</t>
   </si>
   <si>
     <t>LP-052487</t>
@@ -656,12 +656,12 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -716,7 +716,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
@@ -746,57 +746,57 @@
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
@@ -806,12 +806,12 @@
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
@@ -821,27 +821,27 @@
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
@@ -851,27 +851,27 @@
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
@@ -896,17 +896,17 @@
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
@@ -916,22 +916,22 @@
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
@@ -941,7 +941,7 @@
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
@@ -951,67 +951,67 @@
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used: finish lp and om bots
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs - deitado.xlsx
+++ b/08 - Excels/Open-LPs - deitado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3D5295-EFE7-41D4-99C5-BD27718B2F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3AA41A-18CE-47ED-B185-9E18BDA2F515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,237 +20,174 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
   <si>
     <t>LP</t>
   </si>
   <si>
-    <t>LP-039759</t>
-  </si>
-  <si>
-    <t>LP-040769</t>
-  </si>
-  <si>
-    <t>LP-047128</t>
-  </si>
-  <si>
-    <t>LP-047983</t>
-  </si>
-  <si>
-    <t>LP-049262</t>
-  </si>
-  <si>
-    <t>LP-049405</t>
-  </si>
-  <si>
-    <t>LP-050001</t>
-  </si>
-  <si>
-    <t>LP-050381</t>
-  </si>
-  <si>
-    <t>LP-050617</t>
-  </si>
-  <si>
-    <t>LP-051070</t>
-  </si>
-  <si>
-    <t>LP-051164</t>
-  </si>
-  <si>
-    <t>LP-051191</t>
-  </si>
-  <si>
-    <t>LP-051216</t>
-  </si>
-  <si>
-    <t>LP-051223</t>
-  </si>
-  <si>
-    <t>LP-051233</t>
-  </si>
-  <si>
-    <t>LP-051226</t>
-  </si>
-  <si>
-    <t>LP-051320</t>
-  </si>
-  <si>
-    <t>LP-051497</t>
-  </si>
-  <si>
-    <t>LP-051624</t>
-  </si>
-  <si>
-    <t>LP-051680</t>
-  </si>
-  <si>
-    <t>LP-051682</t>
-  </si>
-  <si>
-    <t>LP-051635</t>
-  </si>
-  <si>
-    <t>LP-051709</t>
-  </si>
-  <si>
-    <t>LP-051745</t>
-  </si>
-  <si>
-    <t>LP-051746</t>
-  </si>
-  <si>
-    <t>LP-051749</t>
-  </si>
-  <si>
-    <t>LP-051750</t>
-  </si>
-  <si>
-    <t>LP-051883</t>
-  </si>
-  <si>
-    <t>LP-051884</t>
-  </si>
-  <si>
-    <t>LP-051887</t>
-  </si>
-  <si>
-    <t>LP-051904</t>
-  </si>
-  <si>
-    <t>LP-051905</t>
-  </si>
-  <si>
-    <t>LP-051907</t>
-  </si>
-  <si>
-    <t>LP-051908</t>
-  </si>
-  <si>
-    <t>LP-051909</t>
-  </si>
-  <si>
-    <t>LP-051910</t>
-  </si>
-  <si>
-    <t>LP-052008</t>
-  </si>
-  <si>
-    <t>LP-052017</t>
-  </si>
-  <si>
-    <t>LP-052018</t>
-  </si>
-  <si>
-    <t>LP-052028</t>
-  </si>
-  <si>
-    <t>LP-052029</t>
-  </si>
-  <si>
-    <t>LP-052030</t>
-  </si>
-  <si>
-    <t>LP-052108</t>
-  </si>
-  <si>
-    <t>LP-052109</t>
-  </si>
-  <si>
-    <t>LP-052136</t>
-  </si>
-  <si>
-    <t>LP-052153</t>
-  </si>
-  <si>
-    <t>LP-052152</t>
-  </si>
-  <si>
-    <t>LP-052212</t>
-  </si>
-  <si>
-    <t>LP-052214</t>
-  </si>
-  <si>
-    <t>LP-052480</t>
-  </si>
-  <si>
-    <t>LP-052504</t>
-  </si>
-  <si>
-    <t>LP-052508</t>
-  </si>
-  <si>
-    <t>LP-052509</t>
-  </si>
-  <si>
-    <t>LP-052513</t>
-  </si>
-  <si>
-    <t>LP-052514</t>
-  </si>
-  <si>
-    <t>LP-052572</t>
-  </si>
-  <si>
-    <t>LP-052608</t>
-  </si>
-  <si>
-    <t>LP-052628</t>
+    <t>LP-037756</t>
+  </si>
+  <si>
+    <t>LP-043172</t>
+  </si>
+  <si>
+    <t>LP-046472</t>
+  </si>
+  <si>
+    <t>LP-047850</t>
+  </si>
+  <si>
+    <t>LP-047995</t>
+  </si>
+  <si>
+    <t>LP-048318</t>
+  </si>
+  <si>
+    <t>LP-048321</t>
+  </si>
+  <si>
+    <t>LP-050394</t>
+  </si>
+  <si>
+    <t>LP-050480</t>
+  </si>
+  <si>
+    <t>LP-050592</t>
+  </si>
+  <si>
+    <t>LP-051045</t>
+  </si>
+  <si>
+    <t>LP-051127</t>
+  </si>
+  <si>
+    <t>LP-051410</t>
+  </si>
+  <si>
+    <t>LP-051441</t>
+  </si>
+  <si>
+    <t>LP-051496</t>
+  </si>
+  <si>
+    <t>LP-051515</t>
+  </si>
+  <si>
+    <t>LP-051547</t>
+  </si>
+  <si>
+    <t>LP-051590</t>
+  </si>
+  <si>
+    <t>LP-051773</t>
+  </si>
+  <si>
+    <t>LP-051896</t>
+  </si>
+  <si>
+    <t>LP-051897</t>
+  </si>
+  <si>
+    <t>LP-051898</t>
+  </si>
+  <si>
+    <t>LP-051920</t>
+  </si>
+  <si>
+    <t>LP-051921</t>
+  </si>
+  <si>
+    <t>LP-052027</t>
+  </si>
+  <si>
+    <t>LP-052033</t>
+  </si>
+  <si>
+    <t>LP-052143</t>
+  </si>
+  <si>
+    <t>LP-052144</t>
+  </si>
+  <si>
+    <t>LP-052305</t>
+  </si>
+  <si>
+    <t>LP-052425</t>
+  </si>
+  <si>
+    <t>LP-052428</t>
+  </si>
+  <si>
+    <t>LP-052565</t>
+  </si>
+  <si>
+    <t>LP-052566</t>
+  </si>
+  <si>
+    <t>LP-052567</t>
+  </si>
+  <si>
+    <t>LP-052582</t>
+  </si>
+  <si>
+    <t>LP-052593</t>
+  </si>
+  <si>
+    <t>LP-052594</t>
+  </si>
+  <si>
+    <t>LP-052605</t>
+  </si>
+  <si>
+    <t>LP-052606</t>
+  </si>
+  <si>
+    <t>LP-052607</t>
+  </si>
+  <si>
+    <t>LP-052638</t>
+  </si>
+  <si>
+    <t>LP-052673</t>
+  </si>
+  <si>
+    <t>LP-052685</t>
+  </si>
+  <si>
+    <t>LP-052686</t>
+  </si>
+  <si>
+    <t>LP-052718</t>
+  </si>
+  <si>
+    <t>LP-052777</t>
+  </si>
+  <si>
+    <t>LP-052824</t>
+  </si>
+  <si>
+    <t>LP-053000</t>
+  </si>
+  <si>
+    <t>LP-053131</t>
+  </si>
+  <si>
+    <t>LP-053150</t>
+  </si>
+  <si>
+    <t>LP-053166</t>
+  </si>
+  <si>
+    <t>LP-053279</t>
+  </si>
+  <si>
+    <t>LP-052532</t>
   </si>
   <si>
     <t>LP-052688</t>
   </si>
   <si>
-    <t>LP-052782</t>
-  </si>
-  <si>
-    <t>LP-052861</t>
-  </si>
-  <si>
-    <t>LP-052986</t>
-  </si>
-  <si>
-    <t>LP-049643</t>
-  </si>
-  <si>
-    <t>LP-049688</t>
-  </si>
-  <si>
-    <t>LP-051263</t>
-  </si>
-  <si>
-    <t>LP-051683</t>
-  </si>
-  <si>
-    <t>LP-051903</t>
-  </si>
-  <si>
-    <t>LP-051906</t>
-  </si>
-  <si>
-    <t>LP-052009</t>
-  </si>
-  <si>
-    <t>LP-052031</t>
-  </si>
-  <si>
-    <t>LP-052032</t>
-  </si>
-  <si>
-    <t>LP-052061</t>
-  </si>
-  <si>
-    <t>LP-052093</t>
-  </si>
-  <si>
-    <t>LP-052148</t>
-  </si>
-  <si>
-    <t>LP-052462</t>
-  </si>
-  <si>
-    <t>LP-052487</t>
+    <t>LP-052927</t>
   </si>
 </sst>
 </file>
@@ -613,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A79"/>
+  <dimension ref="A1:A58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -656,362 +593,257 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used: finish LP & OM bot
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs - deitado.xlsx
+++ b/08 - Excels/Open-LPs - deitado.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3AA41A-18CE-47ED-B185-9E18BDA2F515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71982D46-C954-437B-B72F-561F40457461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,174 +20,228 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>LP</t>
   </si>
   <si>
-    <t>LP-037756</t>
-  </si>
-  <si>
-    <t>LP-043172</t>
-  </si>
-  <si>
-    <t>LP-046472</t>
-  </si>
-  <si>
-    <t>LP-047850</t>
-  </si>
-  <si>
-    <t>LP-047995</t>
-  </si>
-  <si>
-    <t>LP-048318</t>
-  </si>
-  <si>
-    <t>LP-048321</t>
-  </si>
-  <si>
-    <t>LP-050394</t>
-  </si>
-  <si>
-    <t>LP-050480</t>
-  </si>
-  <si>
-    <t>LP-050592</t>
-  </si>
-  <si>
-    <t>LP-051045</t>
-  </si>
-  <si>
-    <t>LP-051127</t>
-  </si>
-  <si>
-    <t>LP-051410</t>
-  </si>
-  <si>
-    <t>LP-051441</t>
-  </si>
-  <si>
-    <t>LP-051496</t>
-  </si>
-  <si>
-    <t>LP-051515</t>
-  </si>
-  <si>
-    <t>LP-051547</t>
-  </si>
-  <si>
-    <t>LP-051590</t>
-  </si>
-  <si>
-    <t>LP-051773</t>
-  </si>
-  <si>
-    <t>LP-051896</t>
-  </si>
-  <si>
-    <t>LP-051897</t>
-  </si>
-  <si>
-    <t>LP-051898</t>
-  </si>
-  <si>
-    <t>LP-051920</t>
-  </si>
-  <si>
-    <t>LP-051921</t>
-  </si>
-  <si>
-    <t>LP-052027</t>
-  </si>
-  <si>
-    <t>LP-052033</t>
-  </si>
-  <si>
-    <t>LP-052143</t>
-  </si>
-  <si>
-    <t>LP-052144</t>
-  </si>
-  <si>
-    <t>LP-052305</t>
-  </si>
-  <si>
-    <t>LP-052425</t>
-  </si>
-  <si>
-    <t>LP-052428</t>
-  </si>
-  <si>
-    <t>LP-052565</t>
-  </si>
-  <si>
-    <t>LP-052566</t>
-  </si>
-  <si>
-    <t>LP-052567</t>
-  </si>
-  <si>
-    <t>LP-052582</t>
-  </si>
-  <si>
-    <t>LP-052593</t>
-  </si>
-  <si>
-    <t>LP-052594</t>
-  </si>
-  <si>
-    <t>LP-052605</t>
-  </si>
-  <si>
-    <t>LP-052606</t>
-  </si>
-  <si>
-    <t>LP-052607</t>
-  </si>
-  <si>
-    <t>LP-052638</t>
-  </si>
-  <si>
-    <t>LP-052673</t>
-  </si>
-  <si>
-    <t>LP-052685</t>
-  </si>
-  <si>
-    <t>LP-052686</t>
-  </si>
-  <si>
-    <t>LP-052718</t>
-  </si>
-  <si>
-    <t>LP-052777</t>
-  </si>
-  <si>
-    <t>LP-052824</t>
-  </si>
-  <si>
-    <t>LP-053000</t>
-  </si>
-  <si>
-    <t>LP-053131</t>
-  </si>
-  <si>
-    <t>LP-053150</t>
-  </si>
-  <si>
-    <t>LP-053166</t>
-  </si>
-  <si>
-    <t>LP-053279</t>
+    <t>LP-047619</t>
+  </si>
+  <si>
+    <t>LP-047984</t>
+  </si>
+  <si>
+    <t>LP-047985</t>
+  </si>
+  <si>
+    <t>LP-048486</t>
+  </si>
+  <si>
+    <t>LP-048629</t>
+  </si>
+  <si>
+    <t>LP-050795</t>
+  </si>
+  <si>
+    <t>LP-051176</t>
+  </si>
+  <si>
+    <t>LP-051271</t>
+  </si>
+  <si>
+    <t>LP-051555</t>
+  </si>
+  <si>
+    <t>LP-051556</t>
+  </si>
+  <si>
+    <t>LP-051567</t>
+  </si>
+  <si>
+    <t>LP-051579</t>
+  </si>
+  <si>
+    <t>LP-051744</t>
+  </si>
+  <si>
+    <t>LP-051752</t>
+  </si>
+  <si>
+    <t>LP-051774</t>
+  </si>
+  <si>
+    <t>LP-051985</t>
+  </si>
+  <si>
+    <t>LP-051988</t>
+  </si>
+  <si>
+    <t>LP-051992</t>
+  </si>
+  <si>
+    <t>LP-051996</t>
+  </si>
+  <si>
+    <t>LP-052060</t>
+  </si>
+  <si>
+    <t>LP-052075</t>
+  </si>
+  <si>
+    <t>LP-052079</t>
+  </si>
+  <si>
+    <t>LP-052129</t>
+  </si>
+  <si>
+    <t>LP-052131</t>
+  </si>
+  <si>
+    <t>LP-052145</t>
+  </si>
+  <si>
+    <t>LP-052146</t>
+  </si>
+  <si>
+    <t>LP-052149</t>
+  </si>
+  <si>
+    <t>LP-052150</t>
+  </si>
+  <si>
+    <t>LP-052152</t>
+  </si>
+  <si>
+    <t>LP-052182</t>
+  </si>
+  <si>
+    <t>LP-052289</t>
+  </si>
+  <si>
+    <t>LP-052296</t>
+  </si>
+  <si>
+    <t>LP-052323</t>
+  </si>
+  <si>
+    <t>LP-052343</t>
+  </si>
+  <si>
+    <t>LP-052351</t>
+  </si>
+  <si>
+    <t>LP-052394</t>
+  </si>
+  <si>
+    <t>LP-052395</t>
+  </si>
+  <si>
+    <t>LP-052426</t>
+  </si>
+  <si>
+    <t>LP-052488</t>
+  </si>
+  <si>
+    <t>LP-052489</t>
+  </si>
+  <si>
+    <t>LP-052492</t>
+  </si>
+  <si>
+    <t>LP-052495</t>
+  </si>
+  <si>
+    <t>LP-052525</t>
   </si>
   <si>
     <t>LP-052532</t>
   </si>
   <si>
-    <t>LP-052688</t>
-  </si>
-  <si>
-    <t>LP-052927</t>
+    <t>LP-052548</t>
+  </si>
+  <si>
+    <t>LP-052556</t>
+  </si>
+  <si>
+    <t>LP-052570</t>
+  </si>
+  <si>
+    <t>LP-052571</t>
+  </si>
+  <si>
+    <t>LP-052574</t>
+  </si>
+  <si>
+    <t>LP-052575</t>
+  </si>
+  <si>
+    <t>LP-052584</t>
+  </si>
+  <si>
+    <t>LP-052592</t>
+  </si>
+  <si>
+    <t>LP-052640</t>
+  </si>
+  <si>
+    <t>LP-052641</t>
+  </si>
+  <si>
+    <t>LP-052658</t>
+  </si>
+  <si>
+    <t>LP-052661</t>
+  </si>
+  <si>
+    <t>LP-052672</t>
+  </si>
+  <si>
+    <t>LP-052691</t>
+  </si>
+  <si>
+    <t>LP-052717</t>
+  </si>
+  <si>
+    <t>LP-052758</t>
+  </si>
+  <si>
+    <t>LP-052836</t>
+  </si>
+  <si>
+    <t>LP-052844</t>
+  </si>
+  <si>
+    <t>LP-052856</t>
+  </si>
+  <si>
+    <t>LP-052862</t>
+  </si>
+  <si>
+    <t>LP-052952</t>
+  </si>
+  <si>
+    <t>LP-053191</t>
+  </si>
+  <si>
+    <t>LP-053298</t>
+  </si>
+  <si>
+    <t>LP-053320</t>
+  </si>
+  <si>
+    <t>LP-053327</t>
+  </si>
+  <si>
+    <t>LP-053382</t>
+  </si>
+  <si>
+    <t>LP-053450</t>
+  </si>
+  <si>
+    <t>LP-052583</t>
+  </si>
+  <si>
+    <t>LP-052759</t>
   </si>
 </sst>
 </file>
@@ -550,11 +604,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -718,132 +769,212 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>52</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>